<commit_message>
chore(pages): synchronize frontend updates to docs for GitHub Pages deployment
</commit_message>
<xml_diff>
--- a/docs/outputs/DataExport_REQ_2026_EKS_042_20261011_221106.xlsx
+++ b/docs/outputs/DataExport_REQ_2026_EKS_042_20261011_221106.xlsx
@@ -10,18 +10,25 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA_HASIL" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT_PROVENANCE" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KAMUS_DATA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROFILING_KUALITAS_DATA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DATA_HASIL'!$A$1:$K$36</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="Rp #,##0"/>
+    <numFmt numFmtId="165" formatCode="#,##0 &quot;transaksi&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0 &quot;Kolom&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0 &quot;Atribut&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +44,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,8 +76,95 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00334155"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00334155"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00DC2626"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -79,12 +179,40 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFDF5"/>
+        <bgColor rgb="00ECFDF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -106,11 +234,25 @@
         <color rgb="00E2E8F0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="001E3A8A"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001E3A8A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -122,17 +264,91 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,15 +714,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
@@ -574,20 +790,20 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260924-10009</t>
+          <t>TRX-20260928-10005</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24 19:14:01</t>
+          <t>2026-09-28 15:50:38</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>65000000</v>
+        <v>27500000</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -597,22 +813,22 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>CUST-1001</t>
+          <t>CUST-1036</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Agu*** wan</t>
+          <t>Eko*** tyo</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>317100******8832</t>
+          <t>317456******3873</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>0812****402</t>
+          <t>0812****313</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -622,27 +838,27 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Bandung</t>
+          <t>Tangerang</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260922-10013</t>
+          <t>TRX-20260927-10014</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 16:00:52</t>
+          <t>2026-09-27 13:10:08</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>65000000</v>
+        <v>15000000</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -652,22 +868,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>CUST-1002</t>
+          <t>CUST-1070</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Hen*** aya</t>
+          <t>Bud*** oso</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>317151******1922</t>
+          <t>317835******5188</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>0812****136</t>
+          <t>0812****430</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -684,16 +900,16 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260921-10006</t>
+          <t>TRX-20260925-10011</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-21 21:25:00</t>
+          <t>2026-09-25 20:08:48</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>27500000</v>
+        <v>2500000</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -707,22 +923,22 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>CUST-1072</t>
+          <t>CUST-1063</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Agu*** wan</t>
+          <t>Dew*** ari</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>317820******5853</t>
+          <t>317280******4768</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>0812****109</t>
+          <t>0812****549</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -739,12 +955,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260917-10004</t>
+          <t>TRX-20260924-10007</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-17 17:00:17</t>
+          <t>2026-09-24 17:49:26</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -752,7 +968,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -762,22 +978,22 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>CUST-1056</t>
+          <t>CUST-1073</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Eko*** tyo</t>
+          <t>Dew*** ari</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>317147******6994</t>
+          <t>317868******9166</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>0812****991</t>
+          <t>0812****944</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -787,27 +1003,27 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Semarang</t>
+          <t>Tangerang</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260916-10008</t>
+          <t>TRX-20260920-10026</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-16 12:31:19</t>
+          <t>2026-09-20 08:52:48</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>27500000</v>
+        <v>8900000</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -817,22 +1033,22 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>CUST-1094</t>
+          <t>CUST-1098</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Rin*** ina</t>
+          <t>Sit*** ati</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>317357******3425</t>
+          <t>317973******4170</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>0812****540</t>
+          <t>0812****589</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -842,19 +1058,19 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Tangerang</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260913-10002</t>
+          <t>TRX-20260918-10032</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13 09:58:09</t>
+          <t>2026-09-18 08:03:21</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -862,7 +1078,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -872,7 +1088,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>CUST-1040</t>
+          <t>CUST-1005</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -882,12 +1098,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>317735******1187</t>
+          <t>317769******4097</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>0812****533</t>
+          <t>0812****491</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -897,27 +1113,27 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Bandung</t>
+          <t>Semarang</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260907-10027</t>
+          <t>TRX-20260915-10022</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-07 17:10:27</t>
+          <t>2026-09-15 17:15:27</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>8900000</v>
+        <v>15000000</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>QRIS</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -927,22 +1143,22 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>CUST-1069</t>
+          <t>CUST-1014</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Eko*** tyo</t>
+          <t>Ind*** ata</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>317616******2790</t>
+          <t>317713******7281</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>0812****240</t>
+          <t>0812****953</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -952,23 +1168,23 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Semarang</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260904-10035</t>
+          <t>TRX-20260915-10028</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-04 10:46:23</t>
+          <t>2026-09-15 12:16:43</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>42000000</v>
+        <v>8900000</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -982,7 +1198,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>CUST-1011</t>
+          <t>CUST-1044</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -992,12 +1208,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>317488******4592</t>
+          <t>317419******4579</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>0812****384</t>
+          <t>0812****791</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1007,23 +1223,23 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Semarang</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260831-10020</t>
+          <t>TRX-20260913-10027</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31 11:18:58</t>
+          <t>2026-09-13 10:40:22</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>42000000</v>
+        <v>2500000</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -1037,22 +1253,22 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>CUST-1098</t>
+          <t>CUST-1045</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>May*** ini</t>
+          <t>Hen*** aya</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>317468******4200</t>
+          <t>317505******9450</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>0812****916</t>
+          <t>0812****373</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1062,23 +1278,23 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Semarang</t>
+          <t>Tangerang</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260821-10022</t>
+          <t>TRX-20260909-10008</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-08-21 21:58:53</t>
+          <t>2026-09-09 11:14:24</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>15000000</v>
+        <v>2500000</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -1092,22 +1308,22 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>CUST-1088</t>
+          <t>CUST-1097</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Bam*** nto</t>
+          <t>Ind*** ata</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>317410******7770</t>
+          <t>317709******4072</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>0812****454</t>
+          <t>0812****988</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1117,19 +1333,19 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Tangerang</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260821-10031</t>
+          <t>TRX-20260906-10004</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-08-21 21:31:56</t>
+          <t>2026-09-06 12:30:59</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
@@ -1147,7 +1363,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>CUST-1061</t>
+          <t>CUST-1053</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1157,12 +1373,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>317548******9509</t>
+          <t>317899******8508</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>0812****542</t>
+          <t>0812****583</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1172,23 +1388,23 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Medan</t>
+          <t>Semarang</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260821-10017</t>
+          <t>TRX-20260905-10002</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-08-21 20:35:04</t>
+          <t>2026-09-05 13:28:26</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4750000</v>
+        <v>27500000</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -1202,22 +1418,22 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>CUST-1068</t>
+          <t>CUST-1053</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Bud*** oso</t>
+          <t>Bam*** nto</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>317447******5677</t>
+          <t>317127******5837</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>0812****846</t>
+          <t>0812****873</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1227,27 +1443,27 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Denpasar</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260820-10014</t>
+          <t>TRX-20260904-10024</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-08-20 14:45:45</t>
+          <t>2026-09-04 20:35:32</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>42000000</v>
+        <v>27500000</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1257,22 +1473,22 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>CUST-1009</t>
+          <t>CUST-1093</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Rin*** ina</t>
+          <t>Bam*** nto</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>317832******2743</t>
+          <t>317290******1991</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>0812****795</t>
+          <t>0812****906</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1282,27 +1498,27 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260816-10011</t>
+          <t>TRX-20260829-10017</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-08-16 14:38:55</t>
+          <t>2026-08-29 10:22:08</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>42000000</v>
+        <v>15000000</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1312,22 +1528,22 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>CUST-1055</t>
+          <t>CUST-1013</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Ind*** ata</t>
+          <t>Dew*** ari</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>317808******3348</t>
+          <t>317928******7702</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>0812****353</t>
+          <t>0812****796</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1337,23 +1553,23 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Medan</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260815-10015</t>
+          <t>TRX-20260827-10012</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-08-15 14:09:54</t>
+          <t>2026-08-27 20:02:37</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2500000</v>
+        <v>65000000</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -1367,22 +1583,22 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>CUST-1089</t>
+          <t>CUST-1013</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Agu*** wan</t>
+          <t>Ind*** ata</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>317590******4254</t>
+          <t>317750******6658</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>0812****178</t>
+          <t>0812****273</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1392,27 +1608,27 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Tangerang</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260813-10026</t>
+          <t>TRX-20260826-10016</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-08-13 21:45:56</t>
+          <t>2026-08-26 20:27:48</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>65000000</v>
+        <v>42000000</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1422,7 +1638,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>CUST-1057</t>
+          <t>CUST-1021</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1432,12 +1648,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>317421******5743</t>
+          <t>317812******7903</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>0812****692</t>
+          <t>0812****706</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1454,20 +1670,20 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260813-10029</t>
+          <t>TRX-20260826-10003</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-08-13 14:50:00</t>
+          <t>2026-08-26 19:41:13</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>65000000</v>
+        <v>27500000</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1477,22 +1693,22 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>CUST-1016</t>
+          <t>CUST-1046</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Dew*** ari</t>
+          <t>Bud*** oso</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>317780******8871</t>
+          <t>317534******6629</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>0812****210</t>
+          <t>0812****131</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1502,27 +1718,27 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Denpasar</t>
+          <t>Semarang</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260813-10034</t>
+          <t>TRX-20260826-10009</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-08-13 14:29:33</t>
+          <t>2026-08-26 08:21:22</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>15000000</v>
+        <v>4750000</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>QRIS</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1532,22 +1748,22 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>CUST-1046</t>
+          <t>CUST-1064</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Sit*** ati</t>
+          <t>Bam*** nto</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>317845******9839</t>
+          <t>317634******4735</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>0812****639</t>
+          <t>0812****877</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1557,27 +1773,27 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Denpasar</t>
+          <t>Medan</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260812-10025</t>
+          <t>TRX-20260825-10029</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-08-12 13:17:36</t>
+          <t>2026-08-25 19:38:02</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>42000000</v>
+        <v>8900000</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1587,22 +1803,22 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>CUST-1030</t>
+          <t>CUST-1079</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Bam*** nto</t>
+          <t>Rin*** ina</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>317305******8519</t>
+          <t>317356******9181</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>0812****804</t>
+          <t>0812****285</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1619,20 +1835,20 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260809-10001</t>
+          <t>TRX-20260825-10013</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-08-09 20:11:07</t>
+          <t>2026-08-25 18:22:57</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>4750000</v>
+        <v>8900000</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1642,7 +1858,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>CUST-1041</t>
+          <t>CUST-1057</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1652,12 +1868,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>317818******6427</t>
+          <t>317459******9092</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>0812****503</t>
+          <t>0812****713</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1667,27 +1883,27 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Tangerang</t>
+          <t>Bandung</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260806-10007</t>
+          <t>TRX-20260823-10031</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06 08:02:07</t>
+          <t>2026-08-23 19:31:50</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>65000000</v>
+        <v>42000000</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1697,22 +1913,22 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>CUST-1034</t>
+          <t>CUST-1091</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Hen*** aya</t>
+          <t>Bam*** nto</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>317736******3874</t>
+          <t>317888******1081</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>0812****232</t>
+          <t>0812****375</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1722,27 +1938,27 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Bandung</t>
+          <t>Denpasar</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260805-10010</t>
+          <t>TRX-20260822-10021</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05 17:05:28</t>
+          <t>2026-08-22 13:57:10</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>8900000</v>
+        <v>27500000</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>QRIS</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1752,22 +1968,22 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>CUST-1004</t>
+          <t>CUST-1039</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Bam*** nto</t>
+          <t>Eko*** tyo</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>317541******6177</t>
+          <t>317765******4262</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>0812****505</t>
+          <t>0812****407</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1777,27 +1993,27 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Medan</t>
+          <t>Tangerang</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260802-10019</t>
+          <t>TRX-20260813-10030</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>2026-08-02 18:30:40</t>
+          <t>2026-08-13 10:10:17</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>2500000</v>
+        <v>15000000</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1807,22 +2023,22 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>CUST-1071</t>
+          <t>CUST-1045</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Agu*** wan</t>
+          <t>Hen*** aya</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>317913******2652</t>
+          <t>317109******6218</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>0812****955</t>
+          <t>0812****887</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1832,27 +2048,27 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Semarang</t>
+          <t>Surabaya</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260731-10005</t>
+          <t>TRX-20260812-10034</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>2026-07-31 14:27:22</t>
+          <t>2026-08-12 15:43:08</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>4750000</v>
+        <v>27500000</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1862,22 +2078,22 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>CUST-1068</t>
+          <t>CUST-1025</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Sit*** ati</t>
+          <t>Rin*** ina</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>317426******7005</t>
+          <t>317179******8481</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>0812****780</t>
+          <t>0812****169</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -1887,27 +2103,27 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Bandung</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260729-10018</t>
+          <t>TRX-20260810-10035</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>2026-07-29 13:35:04</t>
+          <t>2026-08-10 21:00:57</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>42000000</v>
+        <v>2500000</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1917,22 +2133,22 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>CUST-1057</t>
+          <t>CUST-1051</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Bud*** oso</t>
+          <t>Bam*** nto</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>317258******2058</t>
+          <t>317791******4360</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>0812****253</t>
+          <t>0812****668</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -1942,27 +2158,27 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Denpasar</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260726-10030</t>
+          <t>TRX-20260809-10033</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>2026-07-26 13:46:54</t>
+          <t>2026-08-09 13:13:06</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>15000000</v>
+        <v>42000000</v>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>QRIS</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1972,22 +2188,22 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>CUST-1007</t>
+          <t>CUST-1004</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Eko*** tyo</t>
+          <t>Agu*** wan</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>317918******9980</t>
+          <t>317667******9605</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>0812****937</t>
+          <t>0812****677</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -1997,23 +2213,23 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Bandung</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260726-10012</t>
+          <t>TRX-20260805-10025</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>2026-07-26 09:40:02</t>
+          <t>2026-08-05 15:35:35</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>15000000</v>
+        <v>65000000</v>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
@@ -2027,22 +2243,22 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>CUST-1097</t>
+          <t>CUST-1060</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>May*** ini</t>
+          <t>Ind*** ata</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>317166******7146</t>
+          <t>317421******9006</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>0812****118</t>
+          <t>0812****819</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2052,27 +2268,27 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Tangerang</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260725-10023</t>
+          <t>TRX-20260805-10019</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2026-07-25 15:38:47</t>
+          <t>2026-08-05 12:37:41</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>8900000</v>
+        <v>15000000</v>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2082,22 +2298,22 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>CUST-1024</t>
+          <t>CUST-1004</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Ind*** ata</t>
+          <t>Dew*** ari</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>317717******5829</t>
+          <t>317216******1301</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>0812****756</t>
+          <t>0812****544</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2107,23 +2323,23 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Medan</t>
+          <t>Denpasar</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260725-10032</t>
+          <t>TRX-20260730-10010</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>2026-07-25 13:25:49</t>
+          <t>2026-07-30 18:06:15</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>4750000</v>
+        <v>27500000</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
@@ -2137,22 +2353,22 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>CUST-1080</t>
+          <t>CUST-1031</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Hen*** aya</t>
+          <t>Rin*** ina</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>317745******3717</t>
+          <t>317103******1223</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>0812****233</t>
+          <t>0812****688</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2162,27 +2378,27 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Tangerang</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260724-10016</t>
+          <t>TRX-20260726-10018</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>2026-07-24 17:22:02</t>
+          <t>2026-07-26 10:55:55</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>27500000</v>
+        <v>15000000</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Credit Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2192,22 +2408,22 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>CUST-1007</t>
+          <t>CUST-1005</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Sit*** ati</t>
+          <t>May*** ini</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>317673******2535</t>
+          <t>317391******3325</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>0812****492</t>
+          <t>0812****705</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2217,27 +2433,27 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Tangerang</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260722-10003</t>
+          <t>TRX-20260723-10020</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>2026-07-22 21:07:37</t>
+          <t>2026-07-23 14:09:50</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>4750000</v>
+        <v>8900000</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2247,22 +2463,22 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>CUST-1088</t>
+          <t>CUST-1083</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Eko*** tyo</t>
+          <t>Sit*** ati</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>317344******9077</t>
+          <t>317342******4355</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>0812****685</t>
+          <t>0812****627</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2272,27 +2488,27 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Bandung</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260710-10033</t>
+          <t>TRX-20260720-10023</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>2026-07-10 12:57:32</t>
+          <t>2026-07-20 08:40:08</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>42000000</v>
+        <v>15000000</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2302,22 +2518,22 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>CUST-1061</t>
+          <t>CUST-1045</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>May*** ini</t>
+          <t>Agu*** wan</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>317958******9100</t>
+          <t>317228******1141</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>0812****505</t>
+          <t>0812****488</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2327,27 +2543,27 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Semarang</t>
+          <t>Medan</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260704-10021</t>
+          <t>TRX-20260716-10001</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>2026-07-04 18:43:14</t>
+          <t>2026-07-16 20:28:35</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>42000000</v>
+        <v>15000000</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>QRIS</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2357,22 +2573,22 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>CUST-1076</t>
+          <t>CUST-1093</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Dew*** ari</t>
+          <t>Ind*** ata</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>317169******9034</t>
+          <t>317908******9573</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>0812****845</t>
+          <t>0812****939</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2382,19 +2598,19 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Jakarta Selatan</t>
+          <t>Surabaya</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260704-10024</t>
+          <t>TRX-20260715-10006</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>2026-07-04 17:17:07</t>
+          <t>2026-07-15 13:12:19</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
@@ -2412,22 +2628,22 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>CUST-1032</t>
+          <t>CUST-1004</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Bam*** nto</t>
+          <t>Eko*** tyo</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>317935******8387</t>
+          <t>317314******9887</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>0812****167</t>
+          <t>0812****248</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2437,23 +2653,23 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Medan</t>
+          <t>Jakarta Selatan</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TRX-20260702-10028</t>
+          <t>TRX-20260701-10015</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>2026-07-02 18:04:50</t>
+          <t>2026-07-01 11:39:27</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>15000000</v>
+        <v>65000000</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
@@ -2467,22 +2683,22 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>CUST-1006</t>
+          <t>CUST-1019</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Eko*** tyo</t>
+          <t>Bud*** oso</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>317957******3691</t>
+          <t>317808******5348</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>0812****740</t>
+          <t>0812****734</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2496,7 +2712,34 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL / SUB-TOTAL</t>
+        </is>
+      </c>
+      <c r="B37" s="6">
+        <f>SUBTOTAL(103, B2:B36)</f>
+        <v/>
+      </c>
+      <c r="C37" s="7">
+        <f>SUBTOTAL(109, C2:C36)</f>
+        <v/>
+      </c>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="6">
+        <f>SUBTOTAL(103, F2:F36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+      <c r="J37" s="8" t="n"/>
+      <c r="K37" s="8" t="n"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:K36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2507,7 +2750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2515,180 +2758,204 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>LOG AUDIT &amp; PROVENANCE DATA PERMOHONAN</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>ID Dokumen Permohonan</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>REQ-2026-EKS-042</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Judul Permohonan</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>SURAT PERMINTAAN DATA DUKUNG PENGAWASAN &amp; AUDIT KEPATUHAN NEGARA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Nama Pemohon</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Bambang Pratama, S.H., M.H.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Unit Kerja / Divisi</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Eksternal Kemenkeu</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Tipe Proses Bisnis</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Keberatan &amp; Banding</t>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Perbendaharaan</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Tujuan Penggunaan Data</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Periode Data</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>01 Juli 2026 s/d 30 September 2026</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Katalog Sumber</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>OpenMetadata Enterprise Catalog (Verified)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Status Verifikasi</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>APPROVED (Agent-Independent-Auditor-v2)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Waktu Verifikasi</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-11T15:11:06.617126+00:00</t>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-13T04:50:31.028664+00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Jumlah Baris Diekstrak</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>35</t>
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Dasar Regulasi PDP</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>UU No. 27/2022 jo. PP No. 33/2026 (LNRI 2026 No. 88)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Proteksi PII / PDP</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Aktif (Masking Dinamis NPWP, NIK, Nama, dan No HP sesuai UU PDP No. 27/2022)</t>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Aktif (Masking Dinamis NPWP, NIK, Nama, dan No HP - Ps. 123 PP 33/2026)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Masa Retensi Wajib</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Maksimal 30 hari kalender sejak penyerahan (Ps. 75 PP 33/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Kewajiban Sanitasi / CoD</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Wajib cryptographic wipe &amp; menerbitkan Certificate of Destruction ke DIKC DJBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Cryptographic Digital Fingerprint</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>SHA256:f8c5fd6a16cf5bdfe120d2d4f044c10df37e093ce7dfd30651ce041fb816166f</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>SHA256:771da77fde0f0113135e87b08f6a4deec3dffef64fb30763eeef6c3552bb9246</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>QUERY SQL YANG DIJALANKAN:</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>-- ====================================================================
--- Query Otomatis Dibuat oleh DataRequest2Agent
+-- Query Otomatis Dibuat oleh DataRequestStudio
 -- Berdasarkan Dokumen: SURAT PERMINTAAN DATA DUKUNG PENGAWASAN &amp; AUDIT KEPATUHAN NEGARA (ID: REQ-2026-EKS-042)
 -- Pemohon: Bambang Pratama, S.H., M.H. (Eksternal Kemenkeu)
 -- Metadata Divalidasi via: OpenMetadata Service CEISA40-PostgreSQL-DWH
@@ -2738,34 +3005,34 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Nama Kolom</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Tipe Data</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Deskripsi Resmi OpenMetadata</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>Klasifikasi PII</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Tabel Sumber</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>nomor_aju</t>
         </is>
@@ -2792,7 +3059,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>nomor_daftar</t>
         </is>
@@ -2819,7 +3086,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>nomor_peb</t>
         </is>
@@ -2846,7 +3113,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>tanggal_daftar</t>
         </is>
@@ -2873,7 +3140,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>tanggal_peb</t>
         </is>
@@ -2900,7 +3167,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>kantor_ekspor</t>
         </is>
@@ -2927,7 +3194,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>kantor_muat</t>
         </is>
@@ -2954,7 +3221,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>kode_kantor</t>
         </is>
@@ -2981,7 +3248,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>npwp_eksportir</t>
         </is>
@@ -3008,7 +3275,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>nama_eksportir</t>
         </is>
@@ -3035,7 +3302,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>alamat_eksportir</t>
         </is>
@@ -3062,7 +3329,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>npwp_ppjk</t>
         </is>
@@ -3089,7 +3356,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>nama_ppjk</t>
         </is>
@@ -3116,7 +3383,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>nama_penerima</t>
         </is>
@@ -3143,7 +3410,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>negara_penerima</t>
         </is>
@@ -3170,7 +3437,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>nama_pembeli</t>
         </is>
@@ -3197,7 +3464,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>negara_pembeli</t>
         </is>
@@ -3224,7 +3491,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>negara_tujuan</t>
         </is>
@@ -3251,7 +3518,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>seri_barang</t>
         </is>
@@ -3278,7 +3545,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>kode_hs</t>
         </is>
@@ -3305,7 +3572,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>uraian_barang</t>
         </is>
@@ -3332,7 +3599,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>jumlah_satuan</t>
         </is>
@@ -3359,7 +3626,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>jenis_satuan</t>
         </is>
@@ -3386,7 +3653,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>netto_barang</t>
         </is>
@@ -3413,7 +3680,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>valuta</t>
         </is>
@@ -3440,7 +3707,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>kurs</t>
         </is>
@@ -3467,7 +3734,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>fob_barang</t>
         </is>
@@ -3494,7 +3761,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>nilai_fob_usd</t>
         </is>
@@ -3521,7 +3788,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>nilai_devisa_idr</t>
         </is>
@@ -3548,7 +3815,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>tarif_bea_keluar</t>
         </is>
@@ -3575,7 +3842,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>bea_keluar_barang</t>
         </is>
@@ -3602,7 +3869,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>pph_ekspor_peb</t>
         </is>
@@ -3629,7 +3896,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>jalur</t>
         </is>
@@ -3656,7 +3923,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>status_pabean</t>
         </is>
@@ -3683,7 +3950,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
@@ -3710,7 +3977,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>nomor_aju</t>
         </is>
@@ -3737,7 +4004,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>nomor_daftar</t>
         </is>
@@ -3764,7 +4031,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>tanggal_daftar</t>
         </is>
@@ -3791,7 +4058,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>kantor_ekspor</t>
         </is>
@@ -3818,7 +4085,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>kantor_muat</t>
         </is>
@@ -3845,7 +4112,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>npwp_eksportir</t>
         </is>
@@ -3872,7 +4139,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>nama_eksportir</t>
         </is>
@@ -3899,7 +4166,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>alamat_eksportir</t>
         </is>
@@ -3926,7 +4193,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="inlineStr">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>npwp_ppjk</t>
         </is>
@@ -3953,7 +4220,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>nama_ppjk</t>
         </is>
@@ -3980,7 +4247,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="inlineStr">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>nama_penerima</t>
         </is>
@@ -4007,7 +4274,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="inlineStr">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>negara_penerima</t>
         </is>
@@ -4034,7 +4301,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="A49" s="15" t="inlineStr">
         <is>
           <t>nama_pembeli</t>
         </is>
@@ -4061,7 +4328,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="inlineStr">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>negara_pembeli</t>
         </is>
@@ -4088,7 +4355,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>negara_tujuan</t>
         </is>
@@ -4115,7 +4382,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="inlineStr">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>seri_barang</t>
         </is>
@@ -4142,7 +4409,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="inlineStr">
+      <c r="A53" s="15" t="inlineStr">
         <is>
           <t>kode_hs</t>
         </is>
@@ -4169,7 +4436,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="inlineStr">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>uraian_barang</t>
         </is>
@@ -4196,7 +4463,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="A55" s="15" t="inlineStr">
         <is>
           <t>jumlah_satuan</t>
         </is>
@@ -4223,7 +4490,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="inlineStr">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>jenis_satuan</t>
         </is>
@@ -4250,7 +4517,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="11" t="inlineStr">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t>netto_barang</t>
         </is>
@@ -4277,7 +4544,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+      <c r="A58" s="15" t="inlineStr">
         <is>
           <t>valuta</t>
         </is>
@@ -4304,7 +4571,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>kurs</t>
         </is>
@@ -4331,7 +4598,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="A60" s="15" t="inlineStr">
         <is>
           <t>fob_barang</t>
         </is>
@@ -4358,7 +4625,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="inlineStr">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t>tarif_bea_keluar</t>
         </is>
@@ -4385,7 +4652,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="inlineStr">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t>bea_keluar_barang</t>
         </is>
@@ -4412,7 +4679,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="inlineStr">
+      <c r="A63" s="15" t="inlineStr">
         <is>
           <t>pph_ekspor_peb</t>
         </is>
@@ -4439,7 +4706,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="11" t="inlineStr">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>jalur</t>
         </is>
@@ -4466,7 +4733,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="11" t="inlineStr">
+      <c r="A65" s="15" t="inlineStr">
         <is>
           <t>status_pabean</t>
         </is>
@@ -4493,7 +4760,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="11" t="inlineStr">
+      <c r="A66" s="15" t="inlineStr">
         <is>
           <t>transaction_id</t>
         </is>
@@ -4520,7 +4787,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="inlineStr">
+      <c r="A67" s="15" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
@@ -4547,7 +4814,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="11" t="inlineStr">
+      <c r="A68" s="15" t="inlineStr">
         <is>
           <t>transaction_date</t>
         </is>
@@ -4574,7 +4841,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="11" t="inlineStr">
+      <c r="A69" s="15" t="inlineStr">
         <is>
           <t>total_amount</t>
         </is>
@@ -4601,7 +4868,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="11" t="inlineStr">
+      <c r="A70" s="15" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -4628,7 +4895,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="11" t="inlineStr">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
@@ -4655,7 +4922,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="11" t="inlineStr">
+      <c r="A72" s="15" t="inlineStr">
         <is>
           <t>npwp_perusahaan</t>
         </is>
@@ -4682,7 +4949,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="11" t="inlineStr">
+      <c r="A73" s="15" t="inlineStr">
         <is>
           <t>nama_perusahaan</t>
         </is>
@@ -4709,7 +4976,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="11" t="inlineStr">
+      <c r="A74" s="15" t="inlineStr">
         <is>
           <t>alamat_domisili</t>
         </is>
@@ -4736,7 +5003,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="11" t="inlineStr">
+      <c r="A75" s="15" t="inlineStr">
         <is>
           <t>nik_penanggung_jawab</t>
         </is>
@@ -4763,7 +5030,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="11" t="inlineStr">
+      <c r="A76" s="15" t="inlineStr">
         <is>
           <t>email_korespondensi</t>
         </is>
@@ -4790,7 +5057,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="11" t="inlineStr">
+      <c r="A77" s="15" t="inlineStr">
         <is>
           <t>nomor_telepon</t>
         </is>
@@ -4817,7 +5084,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="11" t="inlineStr">
+      <c r="A78" s="15" t="inlineStr">
         <is>
           <t>status_registrasi</t>
         </is>
@@ -4844,7 +5111,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="11" t="inlineStr">
+      <c r="A79" s="15" t="inlineStr">
         <is>
           <t>kategori_layanan_aeo</t>
         </is>
@@ -4871,7 +5138,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="11" t="inlineStr">
+      <c r="A80" s="15" t="inlineStr">
         <is>
           <t>tanggal_terdaftar</t>
         </is>
@@ -4900,4 +5167,686 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>PROFILING &amp; METRIK KUALITAS DATA KEPABEANAN (DATA QUALITY SCORECARD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Permohonan: REQ-2026-EKS-042 | Tanggal Analisis: 13 October 2026 | Total Baris: 35 baris</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>SKOR KELENGKAPAN</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL ATRIBUT</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>KOLOM PROTEKSI PDP</t>
+        </is>
+      </c>
+      <c r="K4" s="21" t="inlineStr">
+        <is>
+          <t>STATUS INTEGRITAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="22">
+        <f>AVERAGE(G9:G19)</f>
+        <v/>
+      </c>
+      <c r="E5" s="23">
+        <f>COUNTA(B9:B19)</f>
+        <v/>
+      </c>
+      <c r="H5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K5" s="25" t="inlineStr">
+        <is>
+          <t>100% VALID &amp; VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Nama Atribut / Kolom</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Tipe Data Terdeteksi</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Total Baris</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Terisi (Non-Null)</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Kosong (Null)</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>Rasio Kelengkapan</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>Nilai Unik (Kardinalitas)</t>
+        </is>
+      </c>
+      <c r="I8" s="26" t="inlineStr">
+        <is>
+          <t>Nilai Modus / Terbanyak</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t>Frekuensi</t>
+        </is>
+      </c>
+      <c r="K8" s="26" t="inlineStr">
+        <is>
+          <t>Rentang / Statistik Sebaran</t>
+        </is>
+      </c>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>Status Kepatuhan PDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>transaction_id</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="I9" s="28" t="inlineStr">
+        <is>
+          <t>TRX-20260701-10015</t>
+        </is>
+      </c>
+      <c r="J9" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="31" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 35 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L9" s="27" t="inlineStr">
+        <is>
+          <t>Data Transaksional Standar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>transaction_date</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>Tanggal / Temporal</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="I10" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-01 11:39:27</t>
+        </is>
+      </c>
+      <c r="J10" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="36" t="inlineStr">
+        <is>
+          <t>Rentang: 2026-07-01 11:39:27 s/d 2026-09-28 15:50:38</t>
+        </is>
+      </c>
+      <c r="L10" s="32" t="inlineStr">
+        <is>
+          <t>Data Transaksional Standar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>total_amount</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>Numerik (Integer/Float)</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="F11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" s="28" t="inlineStr">
+        <is>
+          <t>15000000</t>
+        </is>
+      </c>
+      <c r="J11" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="31" t="inlineStr">
+        <is>
+          <t>Min: 2,500,000, Max: 65,000,000, Avg: 21,454,286</t>
+        </is>
+      </c>
+      <c r="L11" s="27" t="inlineStr">
+        <is>
+          <t>Data Transaksional Standar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>payment_method</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D12" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="33" t="inlineStr">
+        <is>
+          <t>Bank Transfer</t>
+        </is>
+      </c>
+      <c r="J12" s="34" t="n">
+        <v>16</v>
+      </c>
+      <c r="K12" s="36" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 3 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L12" s="32" t="inlineStr">
+        <is>
+          <t>Data Transaksional Standar</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="F13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="J13" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="K13" s="31" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 1 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L13" s="27" t="inlineStr">
+        <is>
+          <t>Data Transaksional Standar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="E14" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="34" t="n">
+        <v>27</v>
+      </c>
+      <c r="I14" s="33" t="inlineStr">
+        <is>
+          <t>CUST-1004</t>
+        </is>
+      </c>
+      <c r="J14" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="36" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 27 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L14" s="37" t="inlineStr">
+        <is>
+          <t>Sensitif (Perlu Proteksi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>customer_name_masked</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="E15" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="F15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" s="28" t="inlineStr">
+        <is>
+          <t>Bam*** nto</t>
+        </is>
+      </c>
+      <c r="J15" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" s="31" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 10 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L15" s="38" t="inlineStr">
+        <is>
+          <t>Dimaskir Dinamis (Aman)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>nik_masked</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="I16" s="33" t="inlineStr">
+        <is>
+          <t>317103******1223</t>
+        </is>
+      </c>
+      <c r="J16" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="36" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 35 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L16" s="39" t="inlineStr">
+        <is>
+          <t>Dimaskir Dinamis (Aman)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>phone_masked</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="F17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="I17" s="28" t="inlineStr">
+        <is>
+          <t>0812****131</t>
+        </is>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="31" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 35 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L17" s="38" t="inlineStr">
+        <is>
+          <t>Dimaskir Dinamis (Aman)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>customer_segment</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="E18" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="F18" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="33" t="inlineStr">
+        <is>
+          <t>PRIORITAS</t>
+        </is>
+      </c>
+      <c r="J18" s="34" t="n">
+        <v>35</v>
+      </c>
+      <c r="K18" s="36" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 1 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L18" s="37" t="inlineStr">
+        <is>
+          <t>Sensitif (Perlu Proteksi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>String / Teks Kategoris</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="E19" s="29" t="n">
+        <v>35</v>
+      </c>
+      <c r="F19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="I19" s="28" t="inlineStr">
+        <is>
+          <t>Jakarta Selatan</t>
+        </is>
+      </c>
+      <c r="J19" s="29" t="n">
+        <v>9</v>
+      </c>
+      <c r="K19" s="31" t="inlineStr">
+        <is>
+          <t>Kardinalitas: 7 ragam nilai</t>
+        </is>
+      </c>
+      <c r="L19" s="27" t="inlineStr">
+        <is>
+          <t>Data Transaksional Standar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>